<commit_message>
tambahkan visualisasi data pada tampilan awal
</commit_message>
<xml_diff>
--- a/Rekap.xlsx
+++ b/Rekap.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,17 +25,29 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -56,9 +68,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -434,66 +449,66 @@
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="8"/>
+    <col width="12" customWidth="1" min="6" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="10" max="11"/>
     <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Tanggal Upload</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Nama Pasien</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Tanggal Pemeriksaan</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>ID Pasien</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Umur Pasien</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Jenis Kelamin</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Jenis Pemeriksaan</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Tegangan (kV)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>CTDIvol (mGy)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Total DLP (mGy·cm)</t>
         </is>
@@ -505,7 +520,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-02 21:23:26</t>
+          <t>2026-04-03 09:38:49</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -523,10 +538,8 @@
           <t>680322</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>26 Tahun</t>
-        </is>
+      <c r="F2" t="n">
+        <v>26</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -560,7 +573,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-02 21:24:43</t>
+          <t>2026-04-03 09:39:14</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -578,10 +591,8 @@
           <t>652672</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>26 Tahun</t>
-        </is>
+      <c r="F3" t="n">
+        <v>26</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add delete features and cleanup project files
</commit_message>
<xml_diff>
--- a/Rekap.xlsx
+++ b/Rekap.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -514,112 +514,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-04-03 09:38:49</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>ABDUL RAHMAN. TN</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>02 Feb 2026</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>680322</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>26</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Laki-laki</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>CT KEPALA</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>44.38</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>1250.42</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-04-03 09:39:14</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>PENI FATMAWATI. NY</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>02 Feb 2026</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>652672</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>26</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Perempuan</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>CT KEPALA + KONTRAS</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>44.38</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2586.24</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>